<commit_message>
feat: sync updated laporan hadissss.xls, record TOLAK HOMESTAY cash payments, and update August injected dashboard
</commit_message>
<xml_diff>
--- a/dashboard_agustus_injected.xlsx
+++ b/dashboard_agustus_injected.xlsx
@@ -32219,7 +32219,9 @@
         <f>NamaPelanggan!H215</f>
         <v/>
       </c>
-      <c r="G216" s="120" t="n"/>
+      <c r="G216" s="120" t="n">
+        <v>100000</v>
+      </c>
       <c r="H216" s="120" t="n"/>
       <c r="I216" s="120" t="n"/>
       <c r="J216" s="120" t="n"/>
@@ -32228,14 +32230,8 @@
         <f>IF(SUM(G216:K216)&gt;0,"LUNAS","BELUM LUNAS")</f>
         <v/>
       </c>
-      <c r="M216" s="120" t="n">
-        <v>100000</v>
-      </c>
-      <c r="N216" s="22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="M216" s="120" t="n"/>
+      <c r="N216" s="22" t="n"/>
       <c r="O216" s="6" t="n"/>
       <c r="P216" s="6" t="n"/>
       <c r="Q216" s="6" t="n"/>

</xml_diff>

<commit_message>
feat: migrate database to laporan agustusfix.xls, update August free statuses, and sync injected dashboard
</commit_message>
<xml_diff>
--- a/dashboard_agustus_injected.xlsx
+++ b/dashboard_agustus_injected.xlsx
@@ -35934,14 +35934,8 @@
         <f>IF(SUM(G313:K313)&gt;0,"LUNAS","BELUM LUNAS")</f>
         <v/>
       </c>
-      <c r="M313" s="120" t="n">
-        <v>100000</v>
-      </c>
-      <c r="N313" s="22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="M313" s="120" t="n"/>
+      <c r="N313" s="22" t="n"/>
       <c r="O313" s="6" t="n"/>
       <c r="P313" s="6" t="n"/>
       <c r="Q313" s="6" t="n"/>
@@ -38264,14 +38258,8 @@
         <f>IF(SUM(G374:K374)&gt;0,"LUNAS","BELUM LUNAS")</f>
         <v/>
       </c>
-      <c r="M374" s="120" t="n">
-        <v>100000</v>
-      </c>
-      <c r="N374" s="22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="M374" s="120" t="n"/>
+      <c r="N374" s="22" t="n"/>
       <c r="O374" s="6" t="n"/>
       <c r="P374" s="6" t="n"/>
       <c r="Q374" s="6" t="n"/>
@@ -38306,14 +38294,8 @@
         <f>IF(SUM(G375:K375)&gt;0,"LUNAS","BELUM LUNAS")</f>
         <v/>
       </c>
-      <c r="M375" s="120" t="n">
-        <v>100000</v>
-      </c>
-      <c r="N375" s="22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="M375" s="120" t="n"/>
+      <c r="N375" s="22" t="n"/>
       <c r="O375" s="6" t="n"/>
       <c r="P375" s="6" t="n"/>
       <c r="Q375" s="6" t="n"/>

</xml_diff>